<commit_message>
change the suite name in testng file
</commit_message>
<xml_diff>
--- a/ExcelData/BikeReport.xlsx
+++ b/ExcelData/BikeReport.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="23">
   <si>
     <t>Sr. No.</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>NAME: Bajaj Avenger Street 160 | RATING: 4.4/5 (151 Ratings) | SPECS: 160 cc|45 kmpl|14.79 bhp|156 kg | PRICE: ₹ 1,12,280</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Pulsar N250 | RATING: 4.6/5 (100 Ratings) | SPECS: 249 cc|44 kmpl|24.1 bhp|162 kg | PRICE: ₹ 1,34,758</t>
   </si>
 </sst>
 </file>
@@ -165,7 +168,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -173,7 +176,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -181,7 +184,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -189,7 +192,7 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -205,7 +208,7 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -285,7 +288,7 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -293,7 +296,7 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added 21 to 25 testcase
</commit_message>
<xml_diff>
--- a/ExcelData/BikeReport.xlsx
+++ b/ExcelData/BikeReport.xlsx
@@ -6,14 +6,15 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet_2" r:id="rId4" sheetId="2"/>
-    <sheet name="Sheet_3" r:id="rId5" sheetId="3"/>
+    <sheet name="Sheet_2" r:id="rId7" sheetId="5"/>
+    <sheet name="Sheet_3" r:id="rId5" sheetId="6"/>
+    <sheet name="Sheet_5" r:id="rId6" sheetId="7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="102">
   <si>
     <t>Sr. No</t>
   </si>
@@ -157,6 +158,168 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Bike Name</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>2022 Suzuki Gixxer Single Channel ABS</t>
+  </si>
+  <si>
+    <t>₹ 99,900</t>
+  </si>
+  <si>
+    <t>2017 Suzuki Gixxer Single Channel ABS</t>
+  </si>
+  <si>
+    <t>₹ 50,000</t>
+  </si>
+  <si>
+    <t>2021 Suzuki Gixxer Single Channel ABS - BS4</t>
+  </si>
+  <si>
+    <t>₹ 80,000</t>
+  </si>
+  <si>
+    <t>2014 Suzuki Gixxer Ride Connect</t>
+  </si>
+  <si>
+    <t>₹ 38,000</t>
+  </si>
+  <si>
+    <t>2023 Suzuki Gixxer Ride Connect</t>
+  </si>
+  <si>
+    <t>₹ 90,000</t>
+  </si>
+  <si>
+    <t>2019 Suzuki Gixxer ABS</t>
+  </si>
+  <si>
+    <t>₹ 1.1 Lakh</t>
+  </si>
+  <si>
+    <t>2022 Suzuki Gixxer Standard</t>
+  </si>
+  <si>
+    <t>2017 Suzuki Gixxer Dual Tone Rear Disc</t>
+  </si>
+  <si>
+    <t>₹ 55,000</t>
+  </si>
+  <si>
+    <t>2016 Suzuki Gixxer Dual Tone</t>
+  </si>
+  <si>
+    <t>₹ 45,000</t>
+  </si>
+  <si>
+    <t>₹ 1.4 Lakh</t>
+  </si>
+  <si>
+    <t>2019 Suzuki Gixxer Single Channel ABS</t>
+  </si>
+  <si>
+    <t>₹ 48,000</t>
+  </si>
+  <si>
+    <t>2014 Suzuki Gixxer Single Channel ABS</t>
+  </si>
+  <si>
+    <t>₹ 40,000</t>
+  </si>
+  <si>
+    <t>2020 Suzuki Gixxer Special Edition</t>
+  </si>
+  <si>
+    <t>₹ 1 Lakh</t>
+  </si>
+  <si>
+    <t>2021 Suzuki Gixxer ABS</t>
+  </si>
+  <si>
+    <t>2015 Suzuki Gixxer Single Channel ABS</t>
+  </si>
+  <si>
+    <t>₹ 25,000</t>
+  </si>
+  <si>
+    <t>2018 Suzuki Gixxer Single Channel ABS - BS4</t>
+  </si>
+  <si>
+    <t>2017 Suzuki Gixxer Standard - BS4</t>
+  </si>
+  <si>
+    <t>₹ 42,000</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>2017 Suzuki Gixxer Standard</t>
+  </si>
+  <si>
+    <t>₹ 41,000</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>2015 Suzuki Gixxer Ride Connect</t>
+  </si>
+  <si>
+    <t>₹ 60,000</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>2024 Suzuki Gixxer Ride Connect Special Edition - OBD 2B</t>
+  </si>
+  <si>
+    <t>₹ 1.3 Lakh</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>2021 Suzuki Gixxer Special Edition</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>₹ 95,000</t>
+  </si>
+  <si>
+    <t>2021 Suzuki Gixxer Standard</t>
+  </si>
+  <si>
+    <t>2015 Suzuki Gixxer Standard - BS4</t>
+  </si>
+  <si>
+    <t>₹ 35,000</t>
+  </si>
+  <si>
+    <t>2024 Suzuki Gixxer Ride Connect</t>
+  </si>
+  <si>
+    <t>₹ 1.25 Lakh</t>
+  </si>
+  <si>
+    <t>2024 Suzuki Gixxer Ride Connect [2023-2024]</t>
+  </si>
+  <si>
+    <t>₹ 1.55 Lakh</t>
+  </si>
+  <si>
+    <t>2020 Suzuki Gixxer Standard</t>
   </si>
 </sst>
 </file>
@@ -199,7 +362,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -361,7 +524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -379,7 +542,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>46</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -387,7 +550,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -395,7 +558,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>47</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -403,7 +566,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>47</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -411,7 +574,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -419,7 +582,292 @@
         <v>12</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>47</v>
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
filterBikes sheet name change
</commit_message>
<xml_diff>
--- a/ExcelData/BikeReport.xlsx
+++ b/ExcelData/BikeReport.xlsx
@@ -6,16 +6,17 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet_2" r:id="rId7" sheetId="10"/>
     <sheet name="Sheet_3" r:id="rId5" sheetId="11"/>
     <sheet name="Sheet_4" r:id="rId8" sheetId="12"/>
     <sheet name="Sheet_5" r:id="rId6" sheetId="13"/>
+    <sheet name="Sheet1" r:id="rId9" sheetId="14"/>
+    <sheet name="Sheet_2" r:id="rId7" sheetId="15"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="291">
   <si>
     <t>Sr. No</t>
   </si>
@@ -645,6 +646,249 @@
   </si>
   <si>
     <t>2015 Suzuki Gixxer Single Channel ABS - BS4</t>
+  </si>
+  <si>
+    <t>Rating/Reviews</t>
+  </si>
+  <si>
+    <t>Specs</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar N160</t>
+  </si>
+  <si>
+    <t>4.6/5 (285 Ratings)</t>
+  </si>
+  <si>
+    <t>164.82 cc|51.6 kmpl|15.68 bhp|152 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,14,840</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar NS200</t>
+  </si>
+  <si>
+    <t>4.7/5 (977 Ratings)</t>
+  </si>
+  <si>
+    <t>199.5 cc|36 kmpl|24.13 bhp|158 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,34,162</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar 125</t>
+  </si>
+  <si>
+    <t>4.4/5 (390 Ratings)</t>
+  </si>
+  <si>
+    <t>124.4 cc|50 kmpl|11.64 bhp|140 kg</t>
+  </si>
+  <si>
+    <t>₹ 82,420</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar NS125</t>
+  </si>
+  <si>
+    <t>4.5/5 (160 Ratings)</t>
+  </si>
+  <si>
+    <t>124.45 cc|46.9 kmpl|11.8 bhp|144 kg</t>
+  </si>
+  <si>
+    <t>₹ 92,671</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar NS400Z</t>
+  </si>
+  <si>
+    <t>4.6/5 (106 Ratings)</t>
+  </si>
+  <si>
+    <t>373 cc|32 kmpl|42.41 bhp|174 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,94,061</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar NS160</t>
+  </si>
+  <si>
+    <t>4.6/5 (467 Ratings)</t>
+  </si>
+  <si>
+    <t>160.3 cc|52.2 kmpl|17.03 bhp|152 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,21,837</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar 150</t>
+  </si>
+  <si>
+    <t>4.5/5 (1428 Ratings)</t>
+  </si>
+  <si>
+    <t>149.5 cc|49 kmpl|13.8 bhp|148 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,10,120</t>
+  </si>
+  <si>
+    <t>EV</t>
+  </si>
+  <si>
+    <t>Bajaj Chetak (3.8/5)</t>
+  </si>
+  <si>
+    <t>182 Ratings</t>
+  </si>
+  <si>
+    <t>73 kmph|153 km|3.5 kWh</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar N250</t>
+  </si>
+  <si>
+    <t>4.6/5 (100 Ratings)</t>
+  </si>
+  <si>
+    <t>249 cc|44 kmpl|24.1 bhp|162 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,34,758</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar RS 200</t>
+  </si>
+  <si>
+    <t>4.7/5 (632 Ratings)</t>
+  </si>
+  <si>
+    <t>199.5 cc|35 kmpl|24.1 bhp|167 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,72,857</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar 220 F</t>
+  </si>
+  <si>
+    <t>4.7/5 (92 Ratings)</t>
+  </si>
+  <si>
+    <t>220 cc|40 kmpl|20.11 bhp|160 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,27,481</t>
+  </si>
+  <si>
+    <t>Bajaj Dominar 250</t>
+  </si>
+  <si>
+    <t>4.5/5 (114 Ratings)</t>
+  </si>
+  <si>
+    <t>248.8 cc|35 kmpl|26.63 bhp|180 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,78,273</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar N125</t>
+  </si>
+  <si>
+    <t>4.4/5 (38 Ratings)</t>
+  </si>
+  <si>
+    <t>124.58 cc|60 kmpl|11.83 bhp|125 kg</t>
+  </si>
+  <si>
+    <t>₹ 93,668</t>
+  </si>
+  <si>
+    <t>CNG</t>
+  </si>
+  <si>
+    <t>Bajaj Freedom (4.6/5)</t>
+  </si>
+  <si>
+    <t>117 Ratings</t>
+  </si>
+  <si>
+    <t>125 cc|90 km/kg|9.3 bhp|149 kg</t>
+  </si>
+  <si>
+    <t>Bajaj Chetak C2501 (4.4/5)</t>
+  </si>
+  <si>
+    <t>3 Ratings</t>
+  </si>
+  <si>
+    <t>55 kmph|113 km|108 kg|2.5 kWh</t>
+  </si>
+  <si>
+    <t>Bajaj Avenger Cruise 220</t>
+  </si>
+  <si>
+    <t>4.4/5 (341 Ratings)</t>
+  </si>
+  <si>
+    <t>220 cc|39 kmpl|18.76 bhp|163 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,26,620</t>
+  </si>
+  <si>
+    <t>Bajaj Platina 100</t>
+  </si>
+  <si>
+    <t>4.5/5 (522 Ratings)</t>
+  </si>
+  <si>
+    <t>102 cc|75 kmpl|7.79 bhp|117 kg</t>
+  </si>
+  <si>
+    <t>₹ 66,593</t>
+  </si>
+  <si>
+    <t>Bajaj CT 110</t>
+  </si>
+  <si>
+    <t>4.4/5 (115 Ratings)</t>
+  </si>
+  <si>
+    <t>115.45 cc|70 kmpl|8.48 bhp|127 kg</t>
+  </si>
+  <si>
+    <t>₹ 68,050</t>
+  </si>
+  <si>
+    <t>Bajaj Avenger Street 160</t>
+  </si>
+  <si>
+    <t>4.4/5 (151 Ratings)</t>
+  </si>
+  <si>
+    <t>160 cc|45 kmpl|14.79 bhp|156 kg</t>
+  </si>
+  <si>
+    <t>₹ 1,12,280</t>
+  </si>
+  <si>
+    <t>Bajaj Platina 110</t>
+  </si>
+  <si>
+    <t>4.4/5 (170 Ratings)</t>
+  </si>
+  <si>
+    <t>115.45 cc|70 kmpl|8.48 bhp|119 kg</t>
+  </si>
+  <si>
+    <t>₹ 69,941</t>
   </si>
 </sst>
 </file>
@@ -687,168 +931,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="B15" t="s" s="0">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B7"/>
@@ -1704,4 +1786,470 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>222</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>226</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>238</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>240</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>242</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>253</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>265</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>240</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>269</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>271</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>272</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>273</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>275</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>276</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>287</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>288</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>289</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added wait in TC_12
</commit_message>
<xml_diff>
--- a/ExcelData/BikeReport.xlsx
+++ b/ExcelData/BikeReport.xlsx
@@ -6,16 +6,16 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet_2" r:id="rId7" sheetId="30"/>
-    <sheet name="Sheet_3" r:id="rId9" sheetId="31"/>
-    <sheet name="Sheet_4" r:id="rId8" sheetId="32"/>
-    <sheet name="Sheet_5" r:id="rId6" sheetId="33"/>
+    <sheet name="Sheet_2" r:id="rId7" sheetId="34"/>
+    <sheet name="Sheet_3" r:id="rId9" sheetId="35"/>
+    <sheet name="Sheet_4" r:id="rId8" sheetId="36"/>
+    <sheet name="Sheet_5" r:id="rId6" sheetId="37"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1971" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2222" uniqueCount="219">
   <si>
     <t>Sr. No</t>
   </si>
@@ -714,7 +714,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -876,7 +876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -942,7 +942,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B62"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1448,7 +1448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15.0"/>

</xml_diff>